<commit_message>
Correct 602-0001 and 602-0010 sale unit to bag; clear the review queue
</commit_message>
<xml_diff>
--- a/config/unit_review.xlsx
+++ b/config/unit_review.xlsx
@@ -33,7 +33,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -48,11 +48,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -79,7 +74,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -89,7 +84,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -629,7 +623,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pcs.</t>
+          <t>bag</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -657,22 +651,30 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>sold per 'pcs.' but received per 'bag'</t>
-        </is>
-      </c>
-      <c r="L3" s="4" t="inlineStr">
-        <is>
-          <t>PENDING</t>
+          <t>Sale Unit corrected from 'pcs.' to 'bag' — sold by the bag, and the bag is a parallel unit so the coefficient applies.</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
         </is>
       </c>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Sold per bag (1bag*40pcs / 1bag*10pcs). Confirmed 2026-08-29. 602-0001 implied markup lands on 12.0%, exactly its rule.</t>
+        </is>
+      </c>
       <c r="O3" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -687,7 +689,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>pcs.</t>
+          <t>bag</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -715,22 +717,30 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>sold per 'pcs.' but received per 'bag'</t>
-        </is>
-      </c>
-      <c r="L4" s="4" t="inlineStr">
-        <is>
-          <t>PENDING</t>
+          <t>Sale Unit corrected from 'pcs.' to 'bag' — sold by the bag, and the bag is a parallel unit so the coefficient applies.</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>ACCEPT</t>
         </is>
       </c>
       <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Sold per bag (1bag*40pcs / 1bag*10pcs). Confirmed 2026-08-29. 602-0001 implied markup lands on 12.0%, exactly its rule.</t>
+        </is>
+      </c>
       <c r="O4" t="inlineStr">
         <is>
           <t>2026-08-29</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1182,7 +1192,7 @@
           <t>sale unit is a parallel unit (x4); converted cost 360.25 exceeds the 99.50 selling price (-262% margin) — likely a mis-keyed receipt unit</t>
         </is>
       </c>
-      <c r="L12" s="5" t="inlineStr">
+      <c r="L12" s="4" t="inlineStr">
         <is>
           <t>TREAT_AS</t>
         </is>
@@ -1252,7 +1262,7 @@
           <t>sold per 'pack' but received per 'bag'; sale unit is a parallel unit (x4); converted cost 350.72 exceeds the 99.50 selling price (-252% margin) — likely a mis-keyed receipt unit</t>
         </is>
       </c>
-      <c r="L13" s="5" t="inlineStr">
+      <c r="L13" s="4" t="inlineStr">
         <is>
           <t>TREAT_AS</t>
         </is>
@@ -1322,7 +1332,7 @@
           <t>sold per 'pack' but received per 'bag'; sale unit is a parallel unit (x4); converted cost 368.03 exceeds the 99.50 selling price (-270% margin) — likely a mis-keyed receipt unit</t>
         </is>
       </c>
-      <c r="L14" s="5" t="inlineStr">
+      <c r="L14" s="4" t="inlineStr">
         <is>
           <t>TREAT_AS</t>
         </is>
@@ -1392,7 +1402,7 @@
           <t>sale unit is a parallel unit (x4); converted cost 349.53 exceeds the 98.40 selling price (-255% margin) — likely a mis-keyed receipt unit</t>
         </is>
       </c>
-      <c r="L15" s="5" t="inlineStr">
+      <c r="L15" s="4" t="inlineStr">
         <is>
           <t>TREAT_AS</t>
         </is>

</xml_diff>